<commit_message>
commit - 5 "PR Check"
</commit_message>
<xml_diff>
--- a/qa-artifacts/FoodHub-AI-Test-Coverage.xlsx
+++ b/qa-artifacts/FoodHub-AI-Test-Coverage.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -542,16 +542,116 @@
         <v>User returns to FoodHub and paid order receipt is shown</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>AI-EDGE-007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Contract</v>
+      </c>
+      <c r="C8" t="str">
+        <v>FoodHub Web consumer expects stable /menu and /order contracts</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Consumer/provider API contract drift</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Contract</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Pact verifies GET /menu and POST /order response status, headers, and body shape</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>AI-EDGE-008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Database</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Paid order persists in a real PostgreSQL database</v>
+      </c>
+      <c r="D9" t="str">
+        <v>API returns success but order is not stored</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Integration</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Testcontainers starts PostgreSQL and verifies saved order data can be read back</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>AI-EDGE-009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Load</v>
+      </c>
+      <c r="C10" t="str">
+        <v>API handles repeated browse-and-order traffic</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Performance regression or elevated failure rate under load</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Load</v>
+      </c>
+      <c r="F10" t="str">
+        <v>k6 thresholds pass for p95 latency, HTTP failures, and paid-order failures</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>AI-EDGE-010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Report</v>
+      </c>
+      <c r="C11" t="str">
+        <v>QA report includes functional, contract, database, and load evidence</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Mandatory add-on evidence missing from review artifacts</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Report</v>
+      </c>
+      <c r="F11" t="str">
+        <v>test-report.html shows Dashboard, Integration Testcontainers case, Contract, E2E, and Load metrics</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>AI-EDGE-011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Visual Regression</v>
+      </c>
+      <c r="C12" t="str">
+        <v>UI layout or styling changes unexpectedly</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Checkout UI regressions are missed by functional assertions</v>
+      </c>
+      <c r="E12" t="str">
+        <v>E2E</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Playwright snapshot assertions compare menu-visible, cart-ready, and gateway-ready baselines</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -655,16 +755,118 @@
         <v>Candidate</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>AI-COV-006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Consumer/provider contract regression</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Frontend can break if API fields or status codes change</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Use Pact to verify /menu and successful /order expectations</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Implemented</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>AI-COV-007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Real database persistence</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Mocked persistence can miss PostgreSQL schema or serialization bugs</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Use Testcontainers PostgreSQL to create an order and query it back</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Implemented</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>AI-COV-008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Load-test endpoint hit accounting</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Reviewers need to know how much traffic was generated per endpoint</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Report k6 VUs, iterations, total requests, and /health, /menu, /order hits</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Implemented</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>AI-COV-009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Missing cardId in API order request</v>
+      </c>
+      <c r="C10" t="str">
+        <v>cardId is optional in schema but the checkout may rely on selected-card traceability</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Submit a valid paid order without cardId and verify accepted behavior is intentional</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Candidate</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>AI-COV-010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Testcontainers unavailable in CI</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Real DB tests depend on Docker availability</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Document or gate real DB tests when Docker/Testcontainers cannot start</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Candidate</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>AI-COV-011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Visual regression for checkout UI</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Functional E2E tests may pass even if layout, spacing, or visual hierarchy breaks</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Use Playwright screenshot snapshots for menu-visible, cart-ready, gateway-ready, declined-payment, fake-card, and receipt states</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Partially Implemented</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -751,16 +953,84 @@
         <v>Validate totals across repeated menu item ids</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>AI-DATA-005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>E2E checkout scenario</v>
+      </c>
+      <c r="C6" t="str">
+        <v>createApprovedCheckout()</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Classic Burger, $9.50, CVV 123</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Keep Playwright happy path data centralized and readable</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>AI-DATA-006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>E2E declined card</v>
+      </c>
+      <c r="C7" t="str">
+        <v>createDeclinedPaymentCard()</v>
+      </c>
+      <c r="D7" t="str">
+        <v>declined-card with masked number xxxx-xxxx-xxxx-8911</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Keep payment failure browser data isolated per test</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>AI-DATA-007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>PostgreSQL persisted order</v>
+      </c>
+      <c r="C8" t="str">
+        <v>createOrder([{ menuItemId: 'burger-classic', quantity: 2 }])</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Saved order total 19 with paymentId pay_testcontainers</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Verify real DB persistence and JSONB item serialization</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>AI-DATA-008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>k6 deterministic traffic accounting</v>
+      </c>
+      <c r="C9" t="str">
+        <v>One k6 iteration calls /health, /menu, and /order once</v>
+      </c>
+      <c r="D9" t="str">
+        <v>218 iterations = 654 total API requests</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Make load-test evidence easy to audit</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -814,12 +1084,23 @@
         <v>Review output</v>
       </c>
       <c r="C5" t="str">
-        <v>Look for timeout, selector, network, environment, retry, and ordering patterns</v>
+        <v>Look for timeout, selector, network, Docker/Testcontainers, Pact verifier, k6 threshold, environment, retry, and ordering patterns</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Feed current project context</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Include contract tests, Testcontainers PostgreSQL persistence, k6 load summary, and Playwright E2E artifacts in the AI prompt</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>